<commit_message>
Todo listo para cambio de estructura
</commit_message>
<xml_diff>
--- a/app/Archivos/Template/Template_HRC_D1.xlsx
+++ b/app/Archivos/Template/Template_HRC_D1.xlsx
@@ -517,9 +517,7 @@
           <t>TOTAL s/ BANCOS</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>1852106949</v>
-      </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="C7" s="2" t="n"/>
@@ -546,7 +544,7 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>1852106949</v>
       </c>
     </row>
     <row r="9"/>
@@ -581,9 +579,7 @@
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>1852106949</v>
-      </c>
+      <c r="F12" s="6" t="inlineStr"/>
     </row>
     <row r="13"/>
     <row r="14"/>
@@ -635,16 +631,16 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>PMP1258292</t>
+          <t>PMP1258149</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>6303830</v>
+        <v>25655163</v>
       </c>
       <c r="F19" s="10" t="inlineStr"/>
       <c r="G19" s="10" t="inlineStr"/>
       <c r="H19" s="6" t="n">
-        <v>6303830</v>
+        <v>25655163</v>
       </c>
       <c r="I19" s="11" t="inlineStr"/>
     </row>
@@ -656,16 +652,16 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>PMP1258655</t>
+          <t>PMP1258154</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>17258914</v>
+        <v>2170846</v>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
       <c r="G20" s="10" t="inlineStr"/>
       <c r="H20" s="6" t="n">
-        <v>17258914</v>
+        <v>2170846</v>
       </c>
       <c r="I20" s="11" t="inlineStr"/>
     </row>
@@ -677,16 +673,16 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>PMP1258548</t>
+          <t>PMP1258156</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>12975535</v>
+        <v>4096575</v>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
       <c r="G21" s="10" t="inlineStr"/>
       <c r="H21" s="6" t="n">
-        <v>12975535</v>
+        <v>4096575</v>
       </c>
       <c r="I21" s="11" t="inlineStr"/>
     </row>
@@ -698,16 +694,16 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>PMP1259379</t>
+          <t>PMP1258216</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>98292747</v>
+        <v>37979893</v>
       </c>
       <c r="F22" s="10" t="inlineStr"/>
       <c r="G22" s="10" t="inlineStr"/>
       <c r="H22" s="6" t="n">
-        <v>98292747</v>
+        <v>37979893</v>
       </c>
       <c r="I22" s="11" t="inlineStr"/>
     </row>
@@ -719,16 +715,16 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>PMP1260647</t>
+          <t>PMP1258254</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>78979257</v>
+        <v>5427114</v>
       </c>
       <c r="F23" s="10" t="inlineStr"/>
       <c r="G23" s="10" t="inlineStr"/>
       <c r="H23" s="6" t="n">
-        <v>78979257</v>
+        <v>5427114</v>
       </c>
       <c r="I23" s="11" t="inlineStr"/>
     </row>
@@ -740,16 +736,16 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>PMP1260204</t>
+          <t>PMP1258255</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>45078536</v>
+        <v>38950128</v>
       </c>
       <c r="F24" s="10" t="inlineStr"/>
       <c r="G24" s="10" t="inlineStr"/>
       <c r="H24" s="6" t="n">
-        <v>45078536</v>
+        <v>38950128</v>
       </c>
       <c r="I24" s="11" t="inlineStr"/>
     </row>
@@ -761,16 +757,16 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>PMP1260276</t>
+          <t>PMP1258256</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>23662781</v>
+        <v>33682950</v>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
       <c r="G25" s="10" t="inlineStr"/>
       <c r="H25" s="6" t="n">
-        <v>23662781</v>
+        <v>33682950</v>
       </c>
       <c r="I25" s="11" t="inlineStr"/>
     </row>
@@ -782,16 +778,16 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>PMP1260733</t>
+          <t>PMP1258292</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>21848400</v>
+        <v>6303830</v>
       </c>
       <c r="F26" s="10" t="inlineStr"/>
       <c r="G26" s="10" t="inlineStr"/>
       <c r="H26" s="6" t="n">
-        <v>21848400</v>
+        <v>6303830</v>
       </c>
       <c r="I26" s="11" t="inlineStr"/>
     </row>
@@ -803,16 +799,16 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>PMP1260734</t>
+          <t>PMP1258293</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>29306416</v>
+        <v>78357242</v>
       </c>
       <c r="F27" s="10" t="inlineStr"/>
       <c r="G27" s="10" t="inlineStr"/>
       <c r="H27" s="6" t="n">
-        <v>29306416</v>
+        <v>78357242</v>
       </c>
       <c r="I27" s="11" t="inlineStr"/>
     </row>
@@ -824,16 +820,16 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>PMP1260278</t>
+          <t>PMP1258467</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>29445126</v>
+        <v>5427114</v>
       </c>
       <c r="F28" s="10" t="inlineStr"/>
       <c r="G28" s="10" t="inlineStr"/>
       <c r="H28" s="6" t="n">
-        <v>29445126</v>
+        <v>5427114</v>
       </c>
       <c r="I28" s="11" t="inlineStr"/>
     </row>
@@ -845,16 +841,16 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>PMP1260548</t>
+          <t>PMP1258468</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>27765675</v>
+        <v>41776426</v>
       </c>
       <c r="F29" s="10" t="inlineStr"/>
       <c r="G29" s="10" t="inlineStr"/>
       <c r="H29" s="6" t="n">
-        <v>27765675</v>
+        <v>41776426</v>
       </c>
       <c r="I29" s="11" t="inlineStr"/>
     </row>
@@ -866,16 +862,16 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>PMP1260547</t>
+          <t>PMP1258469</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>32562684</v>
+        <v>5462100</v>
       </c>
       <c r="F30" s="10" t="inlineStr"/>
       <c r="G30" s="10" t="inlineStr"/>
       <c r="H30" s="6" t="n">
-        <v>32562684</v>
+        <v>5462100</v>
       </c>
       <c r="I30" s="11" t="inlineStr"/>
     </row>
@@ -887,16 +883,16 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>PMP1260597</t>
+          <t>PMP1258470</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>34733530</v>
+        <v>8683382</v>
       </c>
       <c r="F31" s="10" t="inlineStr"/>
       <c r="G31" s="10" t="inlineStr"/>
       <c r="H31" s="6" t="n">
-        <v>34733530</v>
+        <v>8683382</v>
       </c>
       <c r="I31" s="11" t="inlineStr"/>
     </row>
@@ -908,16 +904,16 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>PMP1260596</t>
+          <t>PMP1258472</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>83814032</v>
+        <v>23220422</v>
       </c>
       <c r="F32" s="10" t="inlineStr"/>
       <c r="G32" s="10" t="inlineStr"/>
       <c r="H32" s="6" t="n">
-        <v>83814032</v>
+        <v>23220422</v>
       </c>
       <c r="I32" s="11" t="inlineStr"/>
     </row>
@@ -929,16 +925,16 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>PMP1260595</t>
+          <t>PMP1258473</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>41420925</v>
+        <v>6827625</v>
       </c>
       <c r="F33" s="10" t="inlineStr"/>
       <c r="G33" s="10" t="inlineStr"/>
       <c r="H33" s="6" t="n">
-        <v>41420925</v>
+        <v>6827625</v>
       </c>
       <c r="I33" s="11" t="inlineStr"/>
     </row>
@@ -950,16 +946,16 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>PMP1259424</t>
+          <t>PMP1258537</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>5427114</v>
+        <v>14110425</v>
       </c>
       <c r="F34" s="10" t="inlineStr"/>
       <c r="G34" s="10" t="inlineStr"/>
       <c r="H34" s="6" t="n">
-        <v>5427114</v>
+        <v>14110425</v>
       </c>
       <c r="I34" s="11" t="inlineStr"/>
     </row>
@@ -971,16 +967,16 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>PMP1259425</t>
+          <t>PMP1258538</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>33181151</v>
+        <v>8683382</v>
       </c>
       <c r="F35" s="10" t="inlineStr"/>
       <c r="G35" s="10" t="inlineStr"/>
       <c r="H35" s="6" t="n">
-        <v>33181151</v>
+        <v>8683382</v>
       </c>
       <c r="I35" s="11" t="inlineStr"/>
     </row>
@@ -992,16 +988,16 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>PMP1260697</t>
+          <t>PMP1258548</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>91233227</v>
+        <v>12975535</v>
       </c>
       <c r="F36" s="10" t="inlineStr"/>
       <c r="G36" s="10" t="inlineStr"/>
       <c r="H36" s="6" t="n">
-        <v>91233227</v>
+        <v>12975535</v>
       </c>
       <c r="I36" s="11" t="inlineStr"/>
     </row>
@@ -1013,16 +1009,16 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>PMP1260682</t>
+          <t>PMP1258655</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>14565600</v>
+        <v>17258914</v>
       </c>
       <c r="F37" s="10" t="inlineStr"/>
       <c r="G37" s="10" t="inlineStr"/>
       <c r="H37" s="6" t="n">
-        <v>14565600</v>
+        <v>17258914</v>
       </c>
       <c r="I37" s="11" t="inlineStr"/>
     </row>
@@ -1034,16 +1030,16 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>PMP1260681</t>
+          <t>PMP1258681</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>22793879</v>
+        <v>52433082</v>
       </c>
       <c r="F38" s="10" t="inlineStr"/>
       <c r="G38" s="10" t="inlineStr"/>
       <c r="H38" s="6" t="n">
-        <v>22793879</v>
+        <v>52433082</v>
       </c>
       <c r="I38" s="11" t="inlineStr"/>
     </row>
@@ -1055,16 +1051,16 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>PMP1260683</t>
+          <t>PMP1258810</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>63624826</v>
+        <v>39584477</v>
       </c>
       <c r="F39" s="10" t="inlineStr"/>
       <c r="G39" s="10" t="inlineStr"/>
       <c r="H39" s="6" t="n">
-        <v>63624826</v>
+        <v>39584477</v>
       </c>
       <c r="I39" s="11" t="inlineStr"/>
     </row>
@@ -1076,39 +1072,51 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>PMP1261062</t>
+          <t>PMP1259010</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>73484887</v>
+        <v>27160432</v>
       </c>
       <c r="F40" s="10" t="inlineStr"/>
       <c r="G40" s="10" t="inlineStr"/>
       <c r="H40" s="6" t="n">
-        <v>73484887</v>
+        <v>27160432</v>
       </c>
       <c r="I40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuentos no asociados a FC</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>PMP1260166</t>
+          <t>PMP1259010</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>45062325</v>
-      </c>
-      <c r="F41" s="10" t="inlineStr"/>
-      <c r="G41" s="10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
       <c r="H41" s="6" t="n">
-        <v>45062325</v>
-      </c>
-      <c r="I41" s="11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="C42" s="10" t="inlineStr">
@@ -1118,16 +1126,16 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>PMP1260167</t>
+          <t>PMP1259086</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>11939651</v>
+        <v>1628134</v>
       </c>
       <c r="F42" s="10" t="inlineStr"/>
       <c r="G42" s="10" t="inlineStr"/>
       <c r="H42" s="6" t="n">
-        <v>11939651</v>
+        <v>1628134</v>
       </c>
       <c r="I42" s="11" t="inlineStr"/>
     </row>
@@ -1139,16 +1147,16 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>PMP1260168</t>
+          <t>PMP1259087</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>47387323</v>
+        <v>8193150</v>
       </c>
       <c r="F43" s="10" t="inlineStr"/>
       <c r="G43" s="10" t="inlineStr"/>
       <c r="H43" s="6" t="n">
-        <v>47387323</v>
+        <v>8193150</v>
       </c>
       <c r="I43" s="11" t="inlineStr"/>
     </row>
@@ -1160,16 +1168,16 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>PMP1260960</t>
+          <t>PMP1259088</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>10924200</v>
+        <v>17250097</v>
       </c>
       <c r="F44" s="10" t="inlineStr"/>
       <c r="G44" s="10" t="inlineStr"/>
       <c r="H44" s="6" t="n">
-        <v>10924200</v>
+        <v>17250097</v>
       </c>
       <c r="I44" s="11" t="inlineStr"/>
     </row>
@@ -1181,16 +1189,16 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>PMP1260961</t>
+          <t>PMP1259136</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>20623033</v>
+        <v>11939651</v>
       </c>
       <c r="F45" s="10" t="inlineStr"/>
       <c r="G45" s="10" t="inlineStr"/>
       <c r="H45" s="6" t="n">
-        <v>20623033</v>
+        <v>11939651</v>
       </c>
       <c r="I45" s="11" t="inlineStr"/>
     </row>
@@ -1202,16 +1210,16 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>PMP1260962</t>
+          <t>PMP1259137</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>55704424</v>
+        <v>35958825</v>
       </c>
       <c r="F46" s="10" t="inlineStr"/>
       <c r="G46" s="10" t="inlineStr"/>
       <c r="H46" s="6" t="n">
-        <v>55704424</v>
+        <v>35958825</v>
       </c>
       <c r="I46" s="11" t="inlineStr"/>
     </row>
@@ -1223,16 +1231,16 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>PMP1260732</t>
+          <t>PMP1259379</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>79868468</v>
+        <v>98292747</v>
       </c>
       <c r="F47" s="10" t="inlineStr"/>
       <c r="G47" s="10" t="inlineStr"/>
       <c r="H47" s="6" t="n">
-        <v>79868468</v>
+        <v>98292747</v>
       </c>
       <c r="I47" s="11" t="inlineStr"/>
     </row>
@@ -1244,16 +1252,16 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>PMP1258254</t>
+          <t>PMP1259421</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>5427114</v>
+        <v>3256268</v>
       </c>
       <c r="F48" s="10" t="inlineStr"/>
       <c r="G48" s="10" t="inlineStr"/>
       <c r="H48" s="6" t="n">
-        <v>5427114</v>
+        <v>3256268</v>
       </c>
       <c r="I48" s="11" t="inlineStr"/>
     </row>
@@ -1265,16 +1273,16 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>PMP1258255</t>
+          <t>PMP1259422</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>38950128</v>
+        <v>910350</v>
       </c>
       <c r="F49" s="10" t="inlineStr"/>
       <c r="G49" s="10" t="inlineStr"/>
       <c r="H49" s="6" t="n">
-        <v>38950128</v>
+        <v>910350</v>
       </c>
       <c r="I49" s="11" t="inlineStr"/>
     </row>
@@ -1286,39 +1294,51 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>PMP1258256</t>
+          <t>PMP1259423</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
-        <v>33682950</v>
+        <v>22432166</v>
       </c>
       <c r="F50" s="10" t="inlineStr"/>
       <c r="G50" s="10" t="inlineStr"/>
       <c r="H50" s="6" t="n">
-        <v>33682950</v>
+        <v>22432166</v>
       </c>
       <c r="I50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Factura</t>
+          <t>Descuentos no asociados a FC</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>PMP1258216</t>
+          <t>PMP1259423</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>37979893</v>
-      </c>
-      <c r="F51" s="10" t="inlineStr"/>
-      <c r="G51" s="10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
       <c r="H51" s="6" t="n">
-        <v>37979893</v>
-      </c>
-      <c r="I51" s="11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="C52" s="10" t="inlineStr">
@@ -1328,16 +1348,16 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>PMP1259136</t>
+          <t>PMP1259424</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>11939651</v>
+        <v>5427114</v>
       </c>
       <c r="F52" s="10" t="inlineStr"/>
       <c r="G52" s="10" t="inlineStr"/>
       <c r="H52" s="6" t="n">
-        <v>11939651</v>
+        <v>5427114</v>
       </c>
       <c r="I52" s="11" t="inlineStr"/>
     </row>
@@ -1349,16 +1369,16 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>PMP1259137</t>
+          <t>PMP1259425</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>35958825</v>
+        <v>33181151</v>
       </c>
       <c r="F53" s="10" t="inlineStr"/>
       <c r="G53" s="10" t="inlineStr"/>
       <c r="H53" s="6" t="n">
-        <v>35958825</v>
+        <v>33181151</v>
       </c>
       <c r="I53" s="11" t="inlineStr"/>
     </row>
@@ -1370,16 +1390,16 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>PMP1258681</t>
+          <t>PMP1259426</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>52433082</v>
+        <v>19947304</v>
       </c>
       <c r="F54" s="10" t="inlineStr"/>
       <c r="G54" s="10" t="inlineStr"/>
       <c r="H54" s="6" t="n">
-        <v>52433082</v>
+        <v>19947304</v>
       </c>
       <c r="I54" s="11" t="inlineStr"/>
     </row>
@@ -1391,16 +1411,16 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>PMP1258469</t>
+          <t>PMP1259477</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>5462100</v>
+        <v>58694897</v>
       </c>
       <c r="F55" s="10" t="inlineStr"/>
       <c r="G55" s="10" t="inlineStr"/>
       <c r="H55" s="6" t="n">
-        <v>5462100</v>
+        <v>58694897</v>
       </c>
       <c r="I55" s="11" t="inlineStr"/>
     </row>
@@ -1412,16 +1432,16 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>PMP1258470</t>
+          <t>PMP1259614</t>
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>8683382</v>
+        <v>52938835</v>
       </c>
       <c r="F56" s="10" t="inlineStr"/>
       <c r="G56" s="10" t="inlineStr"/>
       <c r="H56" s="6" t="n">
-        <v>8683382</v>
+        <v>52938835</v>
       </c>
       <c r="I56" s="11" t="inlineStr"/>
     </row>
@@ -1433,16 +1453,16 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>PMP1258468</t>
+          <t>PMP1260166</t>
         </is>
       </c>
       <c r="E57" s="6" t="n">
-        <v>41776426</v>
+        <v>45062325</v>
       </c>
       <c r="F57" s="10" t="inlineStr"/>
       <c r="G57" s="10" t="inlineStr"/>
       <c r="H57" s="6" t="n">
-        <v>41776426</v>
+        <v>45062325</v>
       </c>
       <c r="I57" s="11" t="inlineStr"/>
     </row>
@@ -1454,16 +1474,16 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>PMP1259088</t>
+          <t>PMP1260167</t>
         </is>
       </c>
       <c r="E58" s="6" t="n">
-        <v>17250097</v>
+        <v>11939651</v>
       </c>
       <c r="F58" s="10" t="inlineStr"/>
       <c r="G58" s="10" t="inlineStr"/>
       <c r="H58" s="6" t="n">
-        <v>17250097</v>
+        <v>11939651</v>
       </c>
       <c r="I58" s="11" t="inlineStr"/>
     </row>
@@ -1475,16 +1495,16 @@
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>PMP1259087</t>
+          <t>PMP1260168</t>
         </is>
       </c>
       <c r="E59" s="6" t="n">
-        <v>8193150</v>
+        <v>47387323</v>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
       <c r="G59" s="10" t="inlineStr"/>
       <c r="H59" s="6" t="n">
-        <v>8193150</v>
+        <v>47387323</v>
       </c>
       <c r="I59" s="11" t="inlineStr"/>
     </row>
@@ -1496,16 +1516,16 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>PMP1259086</t>
+          <t>PMP1260204</t>
         </is>
       </c>
       <c r="E60" s="6" t="n">
-        <v>1628134</v>
+        <v>45078536</v>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
       <c r="G60" s="10" t="inlineStr"/>
       <c r="H60" s="6" t="n">
-        <v>1628134</v>
+        <v>45078536</v>
       </c>
       <c r="I60" s="11" t="inlineStr"/>
     </row>
@@ -1517,16 +1537,16 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>PMP1258537</t>
+          <t>PMP1260276</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>14110425</v>
+        <v>23662781</v>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
       <c r="G61" s="10" t="inlineStr"/>
       <c r="H61" s="6" t="n">
-        <v>14110425</v>
+        <v>23662781</v>
       </c>
       <c r="I61" s="11" t="inlineStr"/>
     </row>
@@ -1538,16 +1558,16 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>PMP1258810</t>
+          <t>PMP1260278</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>39584477</v>
+        <v>29445126</v>
       </c>
       <c r="F62" s="10" t="inlineStr"/>
       <c r="G62" s="10" t="inlineStr"/>
       <c r="H62" s="6" t="n">
-        <v>39584477</v>
+        <v>29445126</v>
       </c>
       <c r="I62" s="11" t="inlineStr"/>
     </row>
@@ -1559,16 +1579,16 @@
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>PMP1258538</t>
+          <t>PMP1260547</t>
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>8683382</v>
+        <v>32562684</v>
       </c>
       <c r="F63" s="10" t="inlineStr"/>
       <c r="G63" s="10" t="inlineStr"/>
       <c r="H63" s="6" t="n">
-        <v>8683382</v>
+        <v>32562684</v>
       </c>
       <c r="I63" s="11" t="inlineStr"/>
     </row>
@@ -1580,16 +1600,16 @@
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>PMP1258156</t>
+          <t>PMP1260548</t>
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>4096575</v>
+        <v>27765675</v>
       </c>
       <c r="F64" s="10" t="inlineStr"/>
       <c r="G64" s="10" t="inlineStr"/>
       <c r="H64" s="6" t="n">
-        <v>4096575</v>
+        <v>27765675</v>
       </c>
       <c r="I64" s="11" t="inlineStr"/>
     </row>
@@ -1601,16 +1621,16 @@
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>PMP1258154</t>
+          <t>PMP1260595</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>2170846</v>
+        <v>41420925</v>
       </c>
       <c r="F65" s="10" t="inlineStr"/>
       <c r="G65" s="10" t="inlineStr"/>
       <c r="H65" s="6" t="n">
-        <v>2170846</v>
+        <v>41420925</v>
       </c>
       <c r="I65" s="11" t="inlineStr"/>
     </row>
@@ -1622,16 +1642,16 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>PMP1258149</t>
+          <t>PMP1260596</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>25655163</v>
+        <v>83814032</v>
       </c>
       <c r="F66" s="10" t="inlineStr"/>
       <c r="G66" s="10" t="inlineStr"/>
       <c r="H66" s="6" t="n">
-        <v>25655163</v>
+        <v>83814032</v>
       </c>
       <c r="I66" s="11" t="inlineStr"/>
     </row>
@@ -1643,16 +1663,16 @@
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>PMP1259010</t>
+          <t>PMP1260597</t>
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>27160432</v>
+        <v>34733530</v>
       </c>
       <c r="F67" s="10" t="inlineStr"/>
       <c r="G67" s="10" t="inlineStr"/>
       <c r="H67" s="6" t="n">
-        <v>27160432</v>
+        <v>34733530</v>
       </c>
       <c r="I67" s="11" t="inlineStr"/>
     </row>
@@ -1664,16 +1684,16 @@
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>PMP1259477</t>
+          <t>PMP1260647</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>58694897</v>
+        <v>78979257</v>
       </c>
       <c r="F68" s="10" t="inlineStr"/>
       <c r="G68" s="10" t="inlineStr"/>
       <c r="H68" s="6" t="n">
-        <v>58694897</v>
+        <v>78979257</v>
       </c>
       <c r="I68" s="11" t="inlineStr"/>
     </row>
@@ -1685,16 +1705,16 @@
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>PMP1259421</t>
+          <t>PMP1260681</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>3256268</v>
+        <v>22793879</v>
       </c>
       <c r="F69" s="10" t="inlineStr"/>
       <c r="G69" s="10" t="inlineStr"/>
       <c r="H69" s="6" t="n">
-        <v>3256268</v>
+        <v>22793879</v>
       </c>
       <c r="I69" s="11" t="inlineStr"/>
     </row>
@@ -1706,16 +1726,16 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>PMP1259422</t>
+          <t>PMP1260682</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>910350</v>
+        <v>14565600</v>
       </c>
       <c r="F70" s="10" t="inlineStr"/>
       <c r="G70" s="10" t="inlineStr"/>
       <c r="H70" s="6" t="n">
-        <v>910350</v>
+        <v>14565600</v>
       </c>
       <c r="I70" s="11" t="inlineStr"/>
     </row>
@@ -1727,16 +1747,16 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>PMP1259423</t>
+          <t>PMP1260683</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>22432166</v>
+        <v>63624826</v>
       </c>
       <c r="F71" s="10" t="inlineStr"/>
       <c r="G71" s="10" t="inlineStr"/>
       <c r="H71" s="6" t="n">
-        <v>22432166</v>
+        <v>63624826</v>
       </c>
       <c r="I71" s="11" t="inlineStr"/>
     </row>
@@ -1748,16 +1768,16 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>PMP1259614</t>
+          <t>PMP1260697</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>52938835</v>
+        <v>91233227</v>
       </c>
       <c r="F72" s="10" t="inlineStr"/>
       <c r="G72" s="10" t="inlineStr"/>
       <c r="H72" s="6" t="n">
-        <v>52938835</v>
+        <v>91233227</v>
       </c>
       <c r="I72" s="11" t="inlineStr"/>
     </row>
@@ -1769,16 +1789,16 @@
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>PMP1259426</t>
+          <t>PMP1260732</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>19947304</v>
+        <v>79868468</v>
       </c>
       <c r="F73" s="10" t="inlineStr"/>
       <c r="G73" s="10" t="inlineStr"/>
       <c r="H73" s="6" t="n">
-        <v>19947304</v>
+        <v>79868468</v>
       </c>
       <c r="I73" s="11" t="inlineStr"/>
     </row>
@@ -1790,16 +1810,16 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>PMP1258467</t>
+          <t>PMP1260733</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>5427114</v>
+        <v>21848400</v>
       </c>
       <c r="F74" s="10" t="inlineStr"/>
       <c r="G74" s="10" t="inlineStr"/>
       <c r="H74" s="6" t="n">
-        <v>5427114</v>
+        <v>21848400</v>
       </c>
       <c r="I74" s="11" t="inlineStr"/>
     </row>
@@ -1811,16 +1831,16 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>PMP1258473</t>
+          <t>PMP1260734</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>6827625</v>
+        <v>29306416</v>
       </c>
       <c r="F75" s="10" t="inlineStr"/>
       <c r="G75" s="10" t="inlineStr"/>
       <c r="H75" s="6" t="n">
-        <v>6827625</v>
+        <v>29306416</v>
       </c>
       <c r="I75" s="11" t="inlineStr"/>
     </row>
@@ -1832,16 +1852,16 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>PMP1258472</t>
+          <t>PMP1260960</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>23220422</v>
+        <v>10924200</v>
       </c>
       <c r="F76" s="10" t="inlineStr"/>
       <c r="G76" s="10" t="inlineStr"/>
       <c r="H76" s="6" t="n">
-        <v>23220422</v>
+        <v>10924200</v>
       </c>
       <c r="I76" s="11" t="inlineStr"/>
     </row>
@@ -1853,56 +1873,44 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>PMP1258293</t>
+          <t>PMP1260961</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>78357242</v>
+        <v>20623033</v>
       </c>
       <c r="F77" s="10" t="inlineStr"/>
       <c r="G77" s="10" t="inlineStr"/>
       <c r="H77" s="6" t="n">
-        <v>78357242</v>
+        <v>20623033</v>
       </c>
       <c r="I77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Descuentos no asociados a FC</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1260597</t>
+          <t>PMP1260962</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F78" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G78" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
+        <v>55704424</v>
+      </c>
+      <c r="F78" s="10" t="inlineStr"/>
+      <c r="G78" s="10" t="inlineStr"/>
       <c r="H78" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I78" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
+        <v>55704424</v>
+      </c>
+      <c r="I78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>Descuentos no asociados a FC</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
@@ -1911,26 +1919,14 @@
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F79" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G79" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
+        <v>73484887</v>
+      </c>
+      <c r="F79" s="10" t="inlineStr"/>
+      <c r="G79" s="10" t="inlineStr"/>
       <c r="H79" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I79" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
+        <v>73484887</v>
+      </c>
+      <c r="I79" s="11" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="C80" s="10" t="inlineStr">
@@ -1940,7 +1936,7 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>PMP1260962</t>
+          <t>PMP1259426</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
@@ -1973,11 +1969,11 @@
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>PMP1259010</t>
+          <t>PMP1260597</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -1986,11 +1982,11 @@
       </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H81" s="6" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
@@ -2006,11 +2002,11 @@
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>PMP1259423</t>
+          <t>PMP1260962</t>
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
@@ -2019,11 +2015,11 @@
       </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H82" s="6" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
@@ -2039,7 +2035,7 @@
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>PMP1259426</t>
+          <t>PMP1261062</t>
         </is>
       </c>
       <c r="E83" s="6" t="n">

</xml_diff>